<commit_message>
GUI workable demo version
</commit_message>
<xml_diff>
--- a/src/20240922_temp_zf_intestine_1.xlsx
+++ b/src/20240922_temp_zf_intestine_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\其他電腦\My Computer\GlycoMSParser\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9D08DF-32D0-415E-9B0A-48BB10BF7F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{549BC9CE-FC09-4C0A-B077-7CEBC762EB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11565" yWindow="2175" windowWidth="18450" windowHeight="13515" activeTab="1" xr2:uid="{CFD31651-57D7-40EF-BE95-C7417EC3B9A0}"/>
+    <workbookView xWindow="7500" yWindow="2085" windowWidth="18450" windowHeight="10305" activeTab="2" xr2:uid="{CFD31651-57D7-40EF-BE95-C7417EC3B9A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Glycanlist" sheetId="2" r:id="rId1"/>
@@ -621,10 +621,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">peak </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>charge</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -744,9 +740,6 @@
   <si>
     <t>only ion list copied from previous Glypick results w/ validation (20240622)</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Structure</t>
   </si>
   <si>
     <t>H3N4</t>
@@ -885,6 +878,14 @@
   </si>
   <si>
     <t>MS2scan_no</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>peak</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Structure</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1904,7 +1905,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
         <v>37</v>
@@ -2009,7 +2010,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C21" t="s">
         <v>36</v>
@@ -2178,7 +2179,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B26" t="s">
         <v>56</v>
@@ -2930,7 +2931,7 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C48" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D48">
         <f t="shared" ref="D48" si="10">E48+21.9819</f>
@@ -3716,44 +3717,44 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6820557B-6CE2-4FD8-86A4-E2CD52A6D2FD}">
-  <dimension ref="A1:K190"/>
+  <dimension ref="A1:J190"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="B1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D1" t="s">
         <v>144</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>145</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>146</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>147</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>148</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>149</v>
       </c>
-      <c r="I1" t="s">
-        <v>150</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="J1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B2">
         <v>12012</v>
@@ -3765,15 +3766,15 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
+        <v>204</v>
+      </c>
+      <c r="J2" t="s">
         <v>206</v>
       </c>
-      <c r="K2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B3">
         <v>14168</v>
@@ -3785,12 +3786,12 @@
         <v>0</v>
       </c>
       <c r="F3" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B4">
         <v>12180</v>
@@ -3802,12 +3803,12 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B5">
         <v>12333</v>
@@ -3819,12 +3820,12 @@
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B6">
         <v>14318</v>
@@ -3836,12 +3837,12 @@
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B7">
         <v>10595</v>
@@ -3853,12 +3854,12 @@
         <v>0</v>
       </c>
       <c r="F7" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B8">
         <v>16688</v>
@@ -3870,12 +3871,12 @@
         <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B9">
         <v>10914</v>
@@ -3887,12 +3888,12 @@
         <v>0</v>
       </c>
       <c r="F9" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B10">
         <v>10753</v>
@@ -3904,12 +3905,12 @@
         <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B11">
         <v>12636</v>
@@ -3921,12 +3922,12 @@
         <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B12">
         <v>12798</v>
@@ -3938,12 +3939,12 @@
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B13">
         <v>14353</v>
@@ -3955,12 +3956,12 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B14">
         <v>14199</v>
@@ -3972,12 +3973,12 @@
         <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B15">
         <v>12367</v>
@@ -3989,12 +3990,12 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B16">
         <v>13537</v>
@@ -4006,12 +4007,12 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B17">
         <v>14260</v>
@@ -4023,12 +4024,12 @@
         <v>0</v>
       </c>
       <c r="F17" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B18">
         <v>12181</v>
@@ -4040,12 +4041,12 @@
         <v>0</v>
       </c>
       <c r="F18" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B19">
         <v>12332</v>
@@ -4057,12 +4058,12 @@
         <v>0</v>
       </c>
       <c r="F19" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B20">
         <v>14419</v>
@@ -4074,12 +4075,12 @@
         <v>0</v>
       </c>
       <c r="F20" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B21">
         <v>14577</v>
@@ -4091,12 +4092,12 @@
         <v>0</v>
       </c>
       <c r="F21" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B22">
         <v>15628</v>
@@ -4108,12 +4109,12 @@
         <v>0</v>
       </c>
       <c r="F22" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B23">
         <v>15447</v>
@@ -4125,12 +4126,12 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B24">
         <v>19126</v>
@@ -4142,12 +4143,12 @@
         <v>0</v>
       </c>
       <c r="F24" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B25">
         <v>18895</v>
@@ -4159,12 +4160,12 @@
         <v>0</v>
       </c>
       <c r="F25" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B26">
         <v>17499</v>
@@ -4176,12 +4177,12 @@
         <v>0</v>
       </c>
       <c r="F26" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B27">
         <v>17649</v>
@@ -4193,12 +4194,12 @@
         <v>0</v>
       </c>
       <c r="F27" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B28">
         <v>17172</v>
@@ -4210,12 +4211,12 @@
         <v>0</v>
       </c>
       <c r="F28" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B29">
         <v>16060</v>
@@ -4227,12 +4228,12 @@
         <v>0</v>
       </c>
       <c r="F29" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B30">
         <v>15485</v>
@@ -4244,12 +4245,12 @@
         <v>0</v>
       </c>
       <c r="F30" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B31">
         <v>16239</v>
@@ -4261,12 +4262,12 @@
         <v>0</v>
       </c>
       <c r="F31" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B32">
         <v>16204</v>
@@ -4278,12 +4279,12 @@
         <v>0</v>
       </c>
       <c r="F32" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B33">
         <v>15922</v>
@@ -4295,12 +4296,12 @@
         <v>0</v>
       </c>
       <c r="F33" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B34">
         <v>17720</v>
@@ -4312,12 +4313,12 @@
         <v>0</v>
       </c>
       <c r="F34" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B35">
         <v>16094</v>
@@ -4329,12 +4330,12 @@
         <v>0</v>
       </c>
       <c r="F35" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B36">
         <v>17537</v>
@@ -4346,12 +4347,12 @@
         <v>0</v>
       </c>
       <c r="F36" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B37">
         <v>16424</v>
@@ -4363,12 +4364,12 @@
         <v>0</v>
       </c>
       <c r="F37" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B38">
         <v>17353</v>
@@ -4380,12 +4381,12 @@
         <v>0</v>
       </c>
       <c r="F38" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B39">
         <v>19314</v>
@@ -4397,12 +4398,12 @@
         <v>0</v>
       </c>
       <c r="F39" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B40">
         <v>21263</v>
@@ -4414,12 +4415,12 @@
         <v>0</v>
       </c>
       <c r="F40" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B41">
         <v>20896</v>
@@ -4431,12 +4432,12 @@
         <v>0</v>
       </c>
       <c r="F41" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B42">
         <v>19550</v>
@@ -4448,12 +4449,12 @@
         <v>0</v>
       </c>
       <c r="F42" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B43">
         <v>18562</v>
@@ -4465,12 +4466,12 @@
         <v>0</v>
       </c>
       <c r="F43" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B44">
         <v>17392</v>
@@ -4482,12 +4483,12 @@
         <v>0</v>
       </c>
       <c r="F44" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B45">
         <v>17247</v>
@@ -4499,12 +4500,12 @@
         <v>0</v>
       </c>
       <c r="F45" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B46">
         <v>16833</v>
@@ -4516,12 +4517,12 @@
         <v>0</v>
       </c>
       <c r="F46" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B47">
         <v>17205</v>
@@ -4533,12 +4534,12 @@
         <v>0</v>
       </c>
       <c r="F47" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B48">
         <v>18250</v>
@@ -4550,12 +4551,12 @@
         <v>0</v>
       </c>
       <c r="F48" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B49">
         <v>17021</v>
@@ -4567,12 +4568,12 @@
         <v>0</v>
       </c>
       <c r="F49" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B50">
         <v>17020</v>
@@ -4584,12 +4585,12 @@
         <v>0</v>
       </c>
       <c r="F50" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B51">
         <v>18589</v>
@@ -4601,12 +4602,12 @@
         <v>0</v>
       </c>
       <c r="F51" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B52">
         <v>18431</v>
@@ -4618,12 +4619,12 @@
         <v>0</v>
       </c>
       <c r="F52" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B53">
         <v>19211</v>
@@ -4635,12 +4636,12 @@
         <v>0</v>
       </c>
       <c r="F53" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B54">
         <v>19231</v>
@@ -4652,12 +4653,12 @@
         <v>0</v>
       </c>
       <c r="F54" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B55">
         <v>19313</v>
@@ -4669,12 +4670,12 @@
         <v>0</v>
       </c>
       <c r="F55" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B56">
         <v>23988</v>
@@ -4686,12 +4687,12 @@
         <v>0</v>
       </c>
       <c r="F56" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B57">
         <v>23871</v>
@@ -4703,12 +4704,12 @@
         <v>0</v>
       </c>
       <c r="F57" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B58">
         <v>25242</v>
@@ -4720,12 +4721,12 @@
         <v>0</v>
       </c>
       <c r="F58" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B59">
         <v>18066</v>
@@ -4737,12 +4738,12 @@
         <v>0</v>
       </c>
       <c r="F59" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B60">
         <v>17770</v>
@@ -4754,12 +4755,12 @@
         <v>0</v>
       </c>
       <c r="F60" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B61">
         <v>19301</v>
@@ -4771,12 +4772,12 @@
         <v>0</v>
       </c>
       <c r="F61" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B62">
         <v>19409</v>
@@ -4788,12 +4789,12 @@
         <v>0</v>
       </c>
       <c r="F62" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B63">
         <v>19491</v>
@@ -4805,12 +4806,12 @@
         <v>0</v>
       </c>
       <c r="F63" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B64">
         <v>17954</v>
@@ -4822,12 +4823,12 @@
         <v>0</v>
       </c>
       <c r="F64" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B65">
         <v>17882</v>
@@ -4839,12 +4840,12 @@
         <v>0</v>
       </c>
       <c r="F65" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B66">
         <v>24039</v>
@@ -4856,12 +4857,12 @@
         <v>0</v>
       </c>
       <c r="F66" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B67">
         <v>20605</v>
@@ -4873,12 +4874,12 @@
         <v>0</v>
       </c>
       <c r="F67" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B68">
         <v>20523</v>
@@ -4890,12 +4891,12 @@
         <v>0</v>
       </c>
       <c r="F68" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B69">
         <v>19425</v>
@@ -4907,12 +4908,12 @@
         <v>0</v>
       </c>
       <c r="F69" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B70">
         <v>19348</v>
@@ -4924,12 +4925,12 @@
         <v>0</v>
       </c>
       <c r="F70" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B71">
         <v>25410</v>
@@ -4941,12 +4942,12 @@
         <v>0</v>
       </c>
       <c r="F71" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B72">
         <v>25012</v>
@@ -4958,12 +4959,12 @@
         <v>0</v>
       </c>
       <c r="F72" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B73">
         <v>19376</v>
@@ -4975,12 +4976,12 @@
         <v>0</v>
       </c>
       <c r="F73" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B74">
         <v>25253</v>
@@ -4992,12 +4993,12 @@
         <v>0</v>
       </c>
       <c r="F74" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B75">
         <v>24797</v>
@@ -5009,12 +5010,12 @@
         <v>0</v>
       </c>
       <c r="F75" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B76">
         <v>26112</v>
@@ -5026,12 +5027,12 @@
         <v>0</v>
       </c>
       <c r="F76" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B77">
         <v>25865</v>
@@ -5043,12 +5044,12 @@
         <v>0</v>
       </c>
       <c r="F77" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B78">
         <v>18942</v>
@@ -5060,12 +5061,12 @@
         <v>0</v>
       </c>
       <c r="F78" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B79">
         <v>18338</v>
@@ -5077,12 +5078,12 @@
         <v>0</v>
       </c>
       <c r="F79" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B80">
         <v>25769</v>
@@ -5094,12 +5095,12 @@
         <v>0</v>
       </c>
       <c r="F80" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B81">
         <v>25000</v>
@@ -5111,12 +5112,12 @@
         <v>0</v>
       </c>
       <c r="F81" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B82">
         <v>25965</v>
@@ -5128,12 +5129,12 @@
         <v>0</v>
       </c>
       <c r="F82" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B83">
         <v>18563</v>
@@ -5145,12 +5146,12 @@
         <v>0</v>
       </c>
       <c r="F83" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B84">
         <v>24766</v>
@@ -5162,12 +5163,12 @@
         <v>0</v>
       </c>
       <c r="F84" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B85">
         <v>18746</v>
@@ -5179,12 +5180,12 @@
         <v>0</v>
       </c>
       <c r="F85" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B86">
         <v>24637</v>
@@ -5196,12 +5197,12 @@
         <v>0</v>
       </c>
       <c r="F86" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B87">
         <v>18612</v>
@@ -5213,12 +5214,12 @@
         <v>0</v>
       </c>
       <c r="F87" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B88">
         <v>25668</v>
@@ -5230,12 +5231,12 @@
         <v>0</v>
       </c>
       <c r="F88" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B89">
         <v>20035</v>
@@ -5247,12 +5248,12 @@
         <v>0</v>
       </c>
       <c r="F89" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B90">
         <v>19532</v>
@@ -5264,12 +5265,12 @@
         <v>0</v>
       </c>
       <c r="F90" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B91">
         <v>20719</v>
@@ -5281,12 +5282,12 @@
         <v>0</v>
       </c>
       <c r="F91" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B92">
         <v>21037</v>
@@ -5298,12 +5299,12 @@
         <v>0</v>
       </c>
       <c r="F92" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B93">
         <v>21276</v>
@@ -5315,12 +5316,12 @@
         <v>0</v>
       </c>
       <c r="F93" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B94">
         <v>20899</v>
@@ -5332,12 +5333,12 @@
         <v>0</v>
       </c>
       <c r="F94" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B95">
         <v>20204</v>
@@ -5349,12 +5350,12 @@
         <v>0</v>
       </c>
       <c r="F95" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B96">
         <v>21345</v>
@@ -5366,12 +5367,12 @@
         <v>0</v>
       </c>
       <c r="F96" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B97">
         <v>20161</v>
@@ -5383,12 +5384,12 @@
         <v>0</v>
       </c>
       <c r="F97" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B98">
         <v>21144</v>
@@ -5400,12 +5401,12 @@
         <v>0</v>
       </c>
       <c r="F98" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B99">
         <v>21080</v>
@@ -5417,12 +5418,12 @@
         <v>0</v>
       </c>
       <c r="F99" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B100">
         <v>20021</v>
@@ -5434,12 +5435,12 @@
         <v>0</v>
       </c>
       <c r="F100" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B101">
         <v>19816</v>
@@ -5451,12 +5452,12 @@
         <v>0</v>
       </c>
       <c r="F101" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B102">
         <v>20008</v>
@@ -5468,12 +5469,12 @@
         <v>0</v>
       </c>
       <c r="F102" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B103">
         <v>19813</v>
@@ -5485,12 +5486,12 @@
         <v>0</v>
       </c>
       <c r="F103" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B104">
         <v>21210</v>
@@ -5502,12 +5503,12 @@
         <v>0</v>
       </c>
       <c r="F104" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B105">
         <v>20877</v>
@@ -5519,12 +5520,12 @@
         <v>0</v>
       </c>
       <c r="F105" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B106">
         <v>27403</v>
@@ -5536,12 +5537,12 @@
         <v>0</v>
       </c>
       <c r="F106" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B107">
         <v>26713</v>
@@ -5553,12 +5554,12 @@
         <v>0</v>
       </c>
       <c r="F107" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B108">
         <v>26313</v>
@@ -5570,12 +5571,12 @@
         <v>0</v>
       </c>
       <c r="F108" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B109">
         <v>27600</v>
@@ -5587,12 +5588,12 @@
         <v>0</v>
       </c>
       <c r="F109" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B110">
         <v>27680</v>
@@ -5604,12 +5605,12 @@
         <v>0</v>
       </c>
       <c r="F110" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B111">
         <v>27891</v>
@@ -5621,12 +5622,12 @@
         <v>0</v>
       </c>
       <c r="F111" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B112">
         <v>26508</v>
@@ -5638,12 +5639,12 @@
         <v>0</v>
       </c>
       <c r="F112" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B113">
         <v>27807</v>
@@ -5655,12 +5656,12 @@
         <v>0</v>
       </c>
       <c r="F113" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B114">
         <v>20797</v>
@@ -5672,12 +5673,12 @@
         <v>0</v>
       </c>
       <c r="F114" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B115">
         <v>26510</v>
@@ -5689,12 +5690,12 @@
         <v>0</v>
       </c>
       <c r="F115" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B116">
         <v>27482</v>
@@ -5706,12 +5707,12 @@
         <v>0</v>
       </c>
       <c r="F116" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B117">
         <v>21567</v>
@@ -5723,12 +5724,12 @@
         <v>0</v>
       </c>
       <c r="F117" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B118">
         <v>26672</v>
@@ -5740,12 +5741,12 @@
         <v>0</v>
       </c>
       <c r="F118" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B119">
         <v>20106</v>
@@ -5757,12 +5758,12 @@
         <v>0</v>
       </c>
       <c r="F119" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B120">
         <v>21328</v>
@@ -5774,12 +5775,12 @@
         <v>0</v>
       </c>
       <c r="F120" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B121">
         <v>20024</v>
@@ -5791,12 +5792,12 @@
         <v>0</v>
       </c>
       <c r="F121" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B122">
         <v>26964</v>
@@ -5808,12 +5809,12 @@
         <v>0</v>
       </c>
       <c r="F122" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B123">
         <v>25730</v>
@@ -5825,12 +5826,12 @@
         <v>0</v>
       </c>
       <c r="F123" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B124">
         <v>31458</v>
@@ -5842,12 +5843,12 @@
         <v>0</v>
       </c>
       <c r="F124" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B125">
         <v>31272</v>
@@ -5859,12 +5860,12 @@
         <v>0</v>
       </c>
       <c r="F125" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B126">
         <v>31457</v>
@@ -5876,12 +5877,12 @@
         <v>0</v>
       </c>
       <c r="F126" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B127">
         <v>30330</v>
@@ -5893,12 +5894,12 @@
         <v>0</v>
       </c>
       <c r="F127" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B128">
         <v>30446</v>
@@ -5910,12 +5911,12 @@
         <v>0</v>
       </c>
       <c r="F128" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B129">
         <v>30292</v>
@@ -5927,12 +5928,12 @@
         <v>0</v>
       </c>
       <c r="F129" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B130">
         <v>30609</v>
@@ -5944,12 +5945,12 @@
         <v>0</v>
       </c>
       <c r="F130" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B131">
         <v>21795</v>
@@ -5961,12 +5962,12 @@
         <v>0</v>
       </c>
       <c r="F131" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B132">
         <v>22173</v>
@@ -5978,12 +5979,12 @@
         <v>0</v>
       </c>
       <c r="F132" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B133">
         <v>20547</v>
@@ -5995,12 +5996,12 @@
         <v>0</v>
       </c>
       <c r="F133" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B134">
         <v>22298</v>
@@ -6012,12 +6013,12 @@
         <v>0</v>
       </c>
       <c r="F134" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B135">
         <v>21991</v>
@@ -6029,12 +6030,12 @@
         <v>0</v>
       </c>
       <c r="F135" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B136">
         <v>20818</v>
@@ -6046,12 +6047,12 @@
         <v>0</v>
       </c>
       <c r="F136" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B137">
         <v>21612</v>
@@ -6063,12 +6064,12 @@
         <v>0</v>
       </c>
       <c r="F137" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B138">
         <v>21119</v>
@@ -6080,12 +6081,12 @@
         <v>0</v>
       </c>
       <c r="F138" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B139">
         <v>30458</v>
@@ -6097,12 +6098,12 @@
         <v>0</v>
       </c>
       <c r="F139" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B140">
         <v>30411</v>
@@ -6114,12 +6115,12 @@
         <v>0</v>
       </c>
       <c r="F140" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B141">
         <v>30333</v>
@@ -6131,12 +6132,12 @@
         <v>0</v>
       </c>
       <c r="F141" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B142">
         <v>31416</v>
@@ -6148,12 +6149,12 @@
         <v>0</v>
       </c>
       <c r="F142" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B143">
         <v>30448</v>
@@ -6165,12 +6166,12 @@
         <v>0</v>
       </c>
       <c r="F143" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B144">
         <v>20858</v>
@@ -6182,12 +6183,12 @@
         <v>0</v>
       </c>
       <c r="F144" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B145">
         <v>20645</v>
@@ -6199,12 +6200,12 @@
         <v>0</v>
       </c>
       <c r="F145" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B146">
         <v>21912</v>
@@ -6216,12 +6217,12 @@
         <v>0</v>
       </c>
       <c r="F146" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B147">
         <v>20616</v>
@@ -6233,12 +6234,12 @@
         <v>0</v>
       </c>
       <c r="F147" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B148">
         <v>21950</v>
@@ -6250,12 +6251,12 @@
         <v>0</v>
       </c>
       <c r="F148" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B149">
         <v>21079</v>
@@ -6267,12 +6268,12 @@
         <v>0</v>
       </c>
       <c r="F149" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B150">
         <v>21746</v>
@@ -6284,12 +6285,12 @@
         <v>0</v>
       </c>
       <c r="F150" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B151">
         <v>22136</v>
@@ -6301,12 +6302,12 @@
         <v>0</v>
       </c>
       <c r="F151" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B152">
         <v>22422</v>
@@ -6318,12 +6319,12 @@
         <v>0</v>
       </c>
       <c r="F152" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B153">
         <v>21732</v>
@@ -6335,12 +6336,12 @@
         <v>0</v>
       </c>
       <c r="F153" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B154">
         <v>23313</v>
@@ -6352,12 +6353,12 @@
         <v>0</v>
       </c>
       <c r="F154" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B155">
         <v>21665</v>
@@ -6369,12 +6370,12 @@
         <v>0</v>
       </c>
       <c r="F155" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B156">
         <v>22102</v>
@@ -6386,12 +6387,12 @@
         <v>0</v>
       </c>
       <c r="F156" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B157">
         <v>22823</v>
@@ -6403,12 +6404,12 @@
         <v>0</v>
       </c>
       <c r="F157" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B158">
         <v>22337</v>
@@ -6420,12 +6421,12 @@
         <v>0</v>
       </c>
       <c r="F158" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B159">
         <v>22618</v>
@@ -6437,12 +6438,12 @@
         <v>0</v>
       </c>
       <c r="F159" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B160">
         <v>23109</v>
@@ -6454,12 +6455,12 @@
         <v>0</v>
       </c>
       <c r="F160" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B161">
         <v>21782</v>
@@ -6471,12 +6472,12 @@
         <v>0</v>
       </c>
       <c r="F161" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B162">
         <v>21580</v>
@@ -6488,12 +6489,12 @@
         <v>0</v>
       </c>
       <c r="F162" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B163">
         <v>22802</v>
@@ -6505,12 +6506,12 @@
         <v>0</v>
       </c>
       <c r="F163" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B164">
         <v>23024</v>
@@ -6522,12 +6523,12 @@
         <v>0</v>
       </c>
       <c r="F164" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B165">
         <v>22149</v>
@@ -6539,12 +6540,12 @@
         <v>0</v>
       </c>
       <c r="F165" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B166">
         <v>22576</v>
@@ -6556,12 +6557,12 @@
         <v>0</v>
       </c>
       <c r="F166" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B167">
         <v>24233</v>
@@ -6573,12 +6574,12 @@
         <v>0</v>
       </c>
       <c r="F167" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B168">
         <v>24067</v>
@@ -6590,12 +6591,12 @@
         <v>0</v>
       </c>
       <c r="F168" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B169">
         <v>23233</v>
@@ -6607,12 +6608,12 @@
         <v>0</v>
       </c>
       <c r="F169" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B170">
         <v>24437</v>
@@ -6624,12 +6625,12 @@
         <v>0</v>
       </c>
       <c r="F170" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B171">
         <v>22575</v>
@@ -6641,12 +6642,12 @@
         <v>0</v>
       </c>
       <c r="F171" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B172">
         <v>22379</v>
@@ -6658,12 +6659,12 @@
         <v>0</v>
       </c>
       <c r="F172" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B173">
         <v>23987</v>
@@ -6675,12 +6676,12 @@
         <v>0</v>
       </c>
       <c r="F173" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B174">
         <v>23433</v>
@@ -6692,12 +6693,12 @@
         <v>0</v>
       </c>
       <c r="F174" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B175">
         <v>22822</v>
@@ -6709,12 +6710,12 @@
         <v>0</v>
       </c>
       <c r="F175" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B176">
         <v>23106</v>
@@ -6726,12 +6727,12 @@
         <v>0</v>
       </c>
       <c r="F176" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B177">
         <v>24847</v>
@@ -6743,12 +6744,12 @@
         <v>0</v>
       </c>
       <c r="F177" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B178">
         <v>23680</v>
@@ -6760,12 +6761,12 @@
         <v>0</v>
       </c>
       <c r="F178" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B179">
         <v>22783</v>
@@ -6777,12 +6778,12 @@
         <v>0</v>
       </c>
       <c r="F179" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B180">
         <v>23870</v>
@@ -6794,12 +6795,12 @@
         <v>0</v>
       </c>
       <c r="F180" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B181">
         <v>22397</v>
@@ -6811,12 +6812,12 @@
         <v>0</v>
       </c>
       <c r="F181" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B182">
         <v>22983</v>
@@ -6828,12 +6829,12 @@
         <v>0</v>
       </c>
       <c r="F182" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B183">
         <v>23825</v>
@@ -6845,12 +6846,12 @@
         <v>0</v>
       </c>
       <c r="F183" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B184">
         <v>23454</v>
@@ -6862,12 +6863,12 @@
         <v>0</v>
       </c>
       <c r="F184" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B185">
         <v>23701</v>
@@ -6879,12 +6880,12 @@
         <v>0</v>
       </c>
       <c r="F185" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B186">
         <v>23063</v>
@@ -6896,12 +6897,12 @@
         <v>0</v>
       </c>
       <c r="F186" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B187">
         <v>22824</v>
@@ -6913,12 +6914,12 @@
         <v>0</v>
       </c>
       <c r="F187" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B188">
         <v>24475</v>
@@ -6930,12 +6931,12 @@
         <v>0</v>
       </c>
       <c r="F188" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B189">
         <v>22495</v>
@@ -6947,12 +6948,12 @@
         <v>0</v>
       </c>
       <c r="F189" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B190">
         <v>22307</v>
@@ -6964,7 +6965,7 @@
         <v>0</v>
       </c>
       <c r="F190" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -6980,28 +6981,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>165</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>166</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>167</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>168</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>169</v>
-      </c>
-      <c r="H1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -8420,7 +8421,7 @@
   <sheetData>
     <row r="3" spans="2:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
@@ -8443,15 +8444,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" t="s">
         <v>155</v>
-      </c>
-      <c r="B1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B2" s="5">
         <v>45557</v>
@@ -8459,48 +8460,48 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B4" t="s">
         <v>159</v>
-      </c>
-      <c r="B4" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="66" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>